<commit_message>
Add root cause, change assessment, change notice, and issue intake workflow
</commit_message>
<xml_diff>
--- a/06_issue_and_change_management/issue-intake-log.xlsx
+++ b/06_issue_and_change_management/issue-intake-log.xlsx
@@ -8,15 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Documents\GitHub\enterprise-data-governance-operating-system\06_issue_and_change_management\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{91E8B4D6-B5C2-409D-BA0D-9B5A40599F2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{080B95A3-2EAF-498F-B99A-4F558C9AF7E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="22695" windowHeight="14476" xr2:uid="{E706066F-CF75-457A-B8A3-0B9DE62A3E5B}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="22695" windowHeight="14476" activeTab="1" xr2:uid="{E706066F-CF75-457A-B8A3-0B9DE62A3E5B}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="3" r:id="rId1"/>
     <sheet name="Issue Log" sheetId="2" r:id="rId2"/>
     <sheet name="Lists" sheetId="1" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Issue Log'!$A$1:$U$5</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -38,11 +41,299 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="89">
+  <si>
+    <t>Issue Intake Log Workbook</t>
+  </si>
+  <si>
+    <t>Purpose</t>
+  </si>
+  <si>
+    <t>Captures data, reporting, access, metadata, and workflow issues in a structured way so they can be triaged, assigned, remediated, and monitored.</t>
+  </si>
+  <si>
+    <t>How to use</t>
+  </si>
+  <si>
+    <t>Log material issues, assign severity and owner, document remediation, and track recurrence and closure.</t>
+  </si>
+  <si>
+    <t>Governance rule</t>
+  </si>
+  <si>
+    <t>Repeated, material, or cross-team issues should not be handled through informal email only; they should be logged and tracked.</t>
+  </si>
+  <si>
+    <t>Severity</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Dimension</t>
+  </si>
+  <si>
+    <t>Output Use Status</t>
+  </si>
+  <si>
+    <t>Recurrence</t>
+  </si>
+  <si>
+    <t>Issue ID</t>
+  </si>
+  <si>
+    <t>Date Identified</t>
+  </si>
+  <si>
+    <t>Reported By</t>
+  </si>
+  <si>
+    <t>Affected Asset / Report / System</t>
+  </si>
+  <si>
+    <t>Issue Summary</t>
+  </si>
+  <si>
+    <t>Quality Dimension</t>
+  </si>
+  <si>
+    <t>Business Impact</t>
+  </si>
+  <si>
+    <t>Assigned Owner</t>
+  </si>
+  <si>
+    <t>Supporting Role</t>
+  </si>
+  <si>
+    <t>Target Resolution Date</t>
+  </si>
+  <si>
+    <t>Root Cause Category</t>
+  </si>
+  <si>
+    <t>Remediation Action</t>
+  </si>
+  <si>
+    <t>Validation Status</t>
+  </si>
+  <si>
+    <t>Closure Date</t>
+  </si>
+  <si>
+    <t>Related Change ID</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>ISS-001</t>
+  </si>
+  <si>
+    <t>N. Adams</t>
+  </si>
+  <si>
+    <t>Data Quality</t>
+  </si>
+  <si>
+    <t>Executive KPI Dashboard</t>
+  </si>
+  <si>
+    <t>KPI total did not reconcile to certified reporting mart</t>
+  </si>
+  <si>
+    <t>Consistency</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Management reporting confidence affected</t>
+  </si>
+  <si>
+    <t>Pause Release</t>
+  </si>
+  <si>
+    <t>Reporting Data Owner</t>
+  </si>
+  <si>
+    <t>Reporting Steward</t>
+  </si>
+  <si>
+    <t>In Remediation</t>
+  </si>
+  <si>
+    <t>Transformation logic defect</t>
+  </si>
+  <si>
+    <t>Correct mapping logic and revalidate downstream totals</t>
+  </si>
+  <si>
+    <t>Pending</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>CHG-004</t>
+  </si>
+  <si>
+    <t>Escalated due to dashboard visibility</t>
+  </si>
+  <si>
+    <t>ISS-002</t>
+  </si>
+  <si>
+    <t>L. Brown</t>
+  </si>
+  <si>
+    <t>Metadata</t>
+  </si>
+  <si>
+    <t>Business Glossary</t>
+  </si>
+  <si>
+    <t>Two teams used conflicting definitions for Active Customer</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>Comparability risk across reporting outputs</t>
+  </si>
+  <si>
+    <t>Continue With Caveat</t>
+  </si>
+  <si>
+    <t>Customer Data Owner</t>
+  </si>
+  <si>
+    <t>Customer Steward</t>
+  </si>
+  <si>
+    <t>Assigned</t>
+  </si>
+  <si>
+    <t>Business rule ambiguity</t>
+  </si>
+  <si>
+    <t>Approve single definition and update glossary</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>CHG-006</t>
+  </si>
+  <si>
+    <t>Requires owner decision</t>
+  </si>
+  <si>
+    <t>ISS-003</t>
+  </si>
+  <si>
+    <t>P. Chen</t>
+  </si>
+  <si>
+    <t>Access</t>
+  </si>
+  <si>
+    <t>Customer Detail Extract</t>
+  </si>
+  <si>
+    <t>Broad export request granted without documented rationale</t>
+  </si>
+  <si>
+    <t>Integrity</t>
+  </si>
+  <si>
+    <t>Sensitive data exposure risk</t>
+  </si>
+  <si>
+    <t>Stop Use</t>
+  </si>
+  <si>
+    <t>Governance Lead</t>
+  </si>
+  <si>
+    <t>In Triage</t>
+  </si>
+  <si>
+    <t>Access workflow breakdown</t>
+  </si>
+  <si>
+    <t>Review access decision and implement stronger logging</t>
+  </si>
+  <si>
+    <t>Potential policy exception</t>
+  </si>
+  <si>
+    <t>ISS-004</t>
+  </si>
+  <si>
+    <t>R. Singh</t>
+  </si>
+  <si>
+    <t>Workflow</t>
+  </si>
+  <si>
+    <t>Monthly Reporting Process</t>
+  </si>
+  <si>
+    <t>Manual adjustment file not version-controlled and approver unclear</t>
+  </si>
+  <si>
+    <t>Accuracy</t>
+  </si>
+  <si>
+    <t>Auditability and release confidence weakened</t>
+  </si>
+  <si>
+    <t>Reporting Manager</t>
+  </si>
+  <si>
+    <t>Open</t>
+  </si>
+  <si>
+    <t>Documentation gap</t>
+  </si>
+  <si>
+    <t>Introduce change notice and traceability requirement</t>
+  </si>
+  <si>
+    <t>CHG-009</t>
+  </si>
+  <si>
+    <t>Linked to recurring month-end pressure</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -69,8 +360,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -385,27 +679,426 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1130DB83-D59A-48A5-8429-A4DB40F04AD3}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="117" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="18" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="135" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10F47D80-A620-4548-A5A9-D653FE56F7AB}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:U5"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.19921875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="30" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="54.86328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.06640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.53125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="37.265625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.06640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.53125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.06640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="21.6640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="23.19921875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="45.53125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16.796875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="13.265625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="12.06640625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.86328125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="32.19921875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B2" s="3">
+        <v>46034</v>
+      </c>
+      <c r="C2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F2" t="s">
+        <v>33</v>
+      </c>
+      <c r="G2" t="s">
+        <v>34</v>
+      </c>
+      <c r="H2" t="s">
+        <v>35</v>
+      </c>
+      <c r="I2" t="s">
+        <v>36</v>
+      </c>
+      <c r="J2" t="s">
+        <v>37</v>
+      </c>
+      <c r="K2" t="s">
+        <v>38</v>
+      </c>
+      <c r="L2" t="s">
+        <v>39</v>
+      </c>
+      <c r="M2" s="3">
+        <v>46037</v>
+      </c>
+      <c r="N2" t="s">
+        <v>40</v>
+      </c>
+      <c r="O2" t="s">
+        <v>41</v>
+      </c>
+      <c r="P2" t="s">
+        <v>42</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>43</v>
+      </c>
+      <c r="S2" t="s">
+        <v>44</v>
+      </c>
+      <c r="T2" t="s">
+        <v>45</v>
+      </c>
+      <c r="U2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B3" s="3">
+        <v>46042</v>
+      </c>
+      <c r="C3" t="s">
+        <v>48</v>
+      </c>
+      <c r="D3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F3" t="s">
+        <v>51</v>
+      </c>
+      <c r="G3" t="s">
+        <v>34</v>
+      </c>
+      <c r="H3" t="s">
+        <v>52</v>
+      </c>
+      <c r="I3" t="s">
+        <v>53</v>
+      </c>
+      <c r="J3" t="s">
+        <v>54</v>
+      </c>
+      <c r="K3" t="s">
+        <v>55</v>
+      </c>
+      <c r="L3" t="s">
+        <v>56</v>
+      </c>
+      <c r="M3" s="3">
+        <v>46049</v>
+      </c>
+      <c r="N3" t="s">
+        <v>57</v>
+      </c>
+      <c r="O3" t="s">
+        <v>58</v>
+      </c>
+      <c r="P3" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>43</v>
+      </c>
+      <c r="S3" t="s">
+        <v>60</v>
+      </c>
+      <c r="T3" t="s">
+        <v>61</v>
+      </c>
+      <c r="U3" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B4" s="3">
+        <v>46054</v>
+      </c>
+      <c r="C4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D4" t="s">
+        <v>65</v>
+      </c>
+      <c r="E4" t="s">
+        <v>66</v>
+      </c>
+      <c r="F4" t="s">
+        <v>67</v>
+      </c>
+      <c r="G4" t="s">
+        <v>68</v>
+      </c>
+      <c r="H4" t="s">
+        <v>35</v>
+      </c>
+      <c r="I4" t="s">
+        <v>69</v>
+      </c>
+      <c r="J4" t="s">
+        <v>70</v>
+      </c>
+      <c r="K4" t="s">
+        <v>55</v>
+      </c>
+      <c r="L4" t="s">
+        <v>71</v>
+      </c>
+      <c r="M4" s="3">
+        <v>46056</v>
+      </c>
+      <c r="N4" t="s">
+        <v>72</v>
+      </c>
+      <c r="O4" t="s">
+        <v>73</v>
+      </c>
+      <c r="P4" t="s">
+        <v>74</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>43</v>
+      </c>
+      <c r="S4" t="s">
+        <v>44</v>
+      </c>
+      <c r="U4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>76</v>
+      </c>
+      <c r="B5" s="3">
+        <v>46064</v>
+      </c>
+      <c r="C5" t="s">
+        <v>77</v>
+      </c>
+      <c r="D5" t="s">
+        <v>78</v>
+      </c>
+      <c r="E5" t="s">
+        <v>79</v>
+      </c>
+      <c r="F5" t="s">
+        <v>80</v>
+      </c>
+      <c r="G5" t="s">
+        <v>81</v>
+      </c>
+      <c r="H5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I5" t="s">
+        <v>82</v>
+      </c>
+      <c r="J5" t="s">
+        <v>54</v>
+      </c>
+      <c r="K5" t="s">
+        <v>83</v>
+      </c>
+      <c r="L5" t="s">
+        <v>39</v>
+      </c>
+      <c r="M5" s="3">
+        <v>46071</v>
+      </c>
+      <c r="N5" t="s">
+        <v>84</v>
+      </c>
+      <c r="O5" t="s">
+        <v>85</v>
+      </c>
+      <c r="P5" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>43</v>
+      </c>
+      <c r="S5" t="s">
+        <v>60</v>
+      </c>
+      <c r="T5" t="s">
+        <v>87</v>
+      </c>
+      <c r="U5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:U5" xr:uid="{10F47D80-A620-4548-A5A9-D653FE56F7AB}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB697DAD-4B24-4A51-A512-EF1D8380B161}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.9296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.46484375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.73046875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.86328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>